<commit_message>
docs(roadmap): sync v1.1 GitHub publication status and revision history
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="R5a2525b6fdd444ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R21ce4443e0da4980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="R3a3925ae34894c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="R09d4732142c34dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="Rc9ab1265f19848b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R5d51ba65d65a48eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="R09c51b484d404879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="Ree2db40d9b3b47b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="Rcfdc96467d2e4132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="R6140d2ae24374924"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R9b6377602a744e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rf6ef999511c54c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="Radbdcb11c0454f5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="R6faa194c34994359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R3781038a41204c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="Rc94ba5ba55dc4b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="Rec772341566e437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R593e43500b8849c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,7 +158,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -317,6 +317,7 @@
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -324,196 +325,196 @@
   <x:dxfs count="29">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCF4E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD3ECEB"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF0FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8EDF4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFE7FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3E4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAD1D1"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAEDF0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCF4E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD3ECEB"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF0FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8EDF4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFE7FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3E4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAD1D1"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAEDF0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCF4E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD3ECEB"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF0FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8EDF4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFE7FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3E4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAD1D1"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAEDF0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3E4"/>
         </x:patternFill>
       </x:fill>
@@ -667,7 +668,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd94695e81f084494"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcdf7acdd81434d59"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -785,7 +786,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RoadmapHistoryTable" displayName="RoadmapHistoryTable" ref="A5:G9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RoadmapHistoryTable" displayName="RoadmapHistoryTable" ref="A5:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Fecha"/>
     <x:tableColumn id="2" name="ID / línea"/>
@@ -4335,7 +4336,7 @@
         <x:v>PROJECT_MANAGEMENT</x:v>
       </x:c>
       <x:c r="U61" s="22" t="str">
-        <x:v>Estado fichero Excel: generado en esta sesión, subida GitHub pendiente hasta commit.</x:v>
+        <x:v>Excel maestro creado y publicado en rama independiente; no está aún en main.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31" customHeight="1">
@@ -4355,13 +4356,13 @@
         <x:v>Sincronizar Excel del roadmap a rama GitHub del proyecto</x:v>
       </x:c>
       <x:c r="F62" s="22" t="str">
-        <x:v>EN_CURSO</x:v>
+        <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="G62" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H62" s="24" t="n">
-        <x:v>0.35</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I62" s="22" t="n">
         <x:v>1</x:v>
@@ -4370,13 +4371,13 @@
         <x:v>TAP-056</x:v>
       </x:c>
       <x:c r="K62" s="22" t="str">
-        <x:v>Ruta versionada y hash remoto del .xlsx</x:v>
+        <x:v>Excel binario y JSON/CSV publicados por Git blob SHA; rama independiente; merge a main pendiente</x:v>
       </x:c>
       <x:c r="L62" s="22" t="str">
-        <x:v>Pendiente GitHub blob SHA</x:v>
+        <x:v>5f8c7610c / Excel blob 85d2f911</x:v>
       </x:c>
       <x:c r="M62" s="22" t="str">
-        <x:v>https://github.com/Extr3sao/bot_crypto</x:v>
+        <x:v>https://github.com/Extr3sao/bot_crypto/tree/project/roadmap-trading-agentic/docs/roadmap</x:v>
       </x:c>
       <x:c r="N62" s="22" t="str">
         <x:v>ChatGPT</x:v>
@@ -4387,13 +4388,15 @@
         <x:v>2026-10-18</x:v>
       </x:c>
       <x:c r="R62" s="28" t="str">
-        <x:v>Publicar Excel + JSON/CSV + README en rama aislada.</x:v>
+        <x:v>Actualizar Excel tras cada nueva fase; valorar PR a main</x:v>
       </x:c>
       <x:c r="S62" s="28" t="str"/>
       <x:c r="T62" s="22" t="str">
         <x:v>PROJECT_MANAGEMENT</x:v>
       </x:c>
-      <x:c r="U62" s="22" t="str"/>
+      <x:c r="U62" s="22" t="str">
+        <x:v>GitHub commit creado y objeto XLSX verificado por Git SHA-1; la integración en main aún no se ha realizado.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="31" customHeight="1">
       <x:c r="A63" s="26" t="str">
@@ -4624,7 +4627,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfad78393388a4850"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe8c59051d284d69"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -5062,7 +5065,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74affbab45014ba5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e944e32fe8450b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5516,7 +5519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raba12b6654684e5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d494c30861048e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6038,7 +6041,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbff36a8a0b0a4928"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c6cc92555a4baa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6377,7 +6380,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R291692a6440a4425"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ef5a268d4b049e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7015,7 +7018,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81ea7187ae4e4a98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46603a9628b47aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7180,6 +7183,29 @@
         <x:v>v1.0</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>ROADMAP-MASTER-001</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>REMOTE_PUBLISHED</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>Excel y espejo JSON/CSV subidos a rama project/roadmap-trading-agentic; hash Git XLSX verificado; se prepara revisión 1.1.</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F10" s="40" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/commit/5f8c7610c052cad019421041cab5b360e7befc4e</x:v>
+      </x:c>
+      <x:c r="G10" s="40" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
@@ -7187,7 +7213,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d91dfe7995495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbf6ff8981204775"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7426,7 +7452,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>Corte de GitHub: 2026-10-18 · Sin beneficios netos demostrados · Paper/Shadow · Sin trading real</x:v>
+        <x:v>Corte GitHub: 2026-10-18 · v1.1 · Rama de gestión publicada · Sin IA real ni rentabilidad demostrada</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -7471,7 +7497,7 @@
       <x:c r="C6" s="48"/>
       <x:c r="E6" s="48" t="n">
         <x:f>COUNTIF(ROADMAP!F6:F65,"VERIFICADO_FOCAL")</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F6" s="48"/>
       <x:c r="H6" s="48" t="n">
@@ -7533,7 +7559,7 @@
       </x:c>
       <x:c r="L11" s="60" t="n">
         <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K11)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
@@ -7575,7 +7601,7 @@
       </x:c>
       <x:c r="L13" s="60" t="n">
         <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K13)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
@@ -7789,6 +7815,6 @@
     <x:mergeCell ref="B31:I33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60e269aea5e848f7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb7fbc5cf864af2"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): refresh v1.2 AI-BOTS-003C pins and record Windows console UX WP
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="R6140d2ae24374924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R9b6377602a744e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rf6ef999511c54c74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="Radbdcb11c0454f5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="R6faa194c34994359"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R3781038a41204c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="Rc94ba5ba55dc4b56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="Rec772341566e437f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R593e43500b8849c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="Rdc0a02fb1c4f495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="Re0ec1f29096d46ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rac41de3505b14ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="R56293e7283804d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="Rdc34eb2ce6924743"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="Rf58241507cc4417f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="R7b7d10902bfa410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="Rcc121c59484a414b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R803f51fd71344b46"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -668,7 +668,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcdf7acdd81434d59"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfaeb489b26294293"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -678,7 +678,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoadmapMasterTable" displayName="RoadmapMasterTable" ref="A5:U65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoadmapMasterTable" displayName="RoadmapMasterTable" ref="A5:U66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Frente / línea"/>
@@ -721,7 +721,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RFCWorkPackagesTable" displayName="RFCWorkPackagesTable" ref="A5:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RFCWorkPackagesTable" displayName="RFCWorkPackagesTable" ref="A5:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="RFC / WP"/>
     <x:tableColumn id="2" name="Área"/>
@@ -737,7 +737,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BlockedItemsTable" displayName="BlockedItemsTable" ref="A5:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BlockedItemsTable" displayName="BlockedItemsTable" ref="A5:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Prio"/>
@@ -767,7 +767,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceRegisterTable" displayName="EvidenceRegisterTable" ref="A5:K20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceRegisterTable" displayName="EvidenceRegisterTable" ref="A5:K21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Fecha"/>
@@ -786,7 +786,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RoadmapHistoryTable" displayName="RoadmapHistoryTable" ref="A5:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RoadmapHistoryTable" displayName="RoadmapHistoryTable" ref="A5:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Fecha"/>
     <x:tableColumn id="2" name="ID / línea"/>
@@ -2253,7 +2253,7 @@
         <x:v>459 tests suites afectadas; 120 checks en 5 escenarios</x:v>
       </x:c>
       <x:c r="L25" s="22" t="str">
-        <x:v>86d4f12 / BLOCK-C FINAL_REPORT</x:v>
+        <x:v>86d4f12 motor · 0841d37 cierre/recibos</x:v>
       </x:c>
       <x:c r="M25" s="22" t="str">
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ai-bots/RFC-AI-BOTS-003/BLOCK-C/FINAL_REPORT.md</x:v>
@@ -2272,7 +2272,7 @@
         <x:v>REPO_REPORT</x:v>
       </x:c>
       <x:c r="U25" s="22" t="str">
-        <x:v>Runtime commit 86d4f12; evidencia publicada hasta eeb0bea.</x:v>
+        <x:v>Gaps OPEN antes de nuevas entradas. Caso sintético sí; datos reales sin gap OPEN &gt;2%. 459 tests focalizados comunicados; sin modelo real. Reproducibilidad de captura revalidada hasta 0841d37.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="31" customHeight="1">
@@ -2310,7 +2310,7 @@
         <x:v>53 mutaciones detectadas / 12 omitidas por diseño</x:v>
       </x:c>
       <x:c r="L26" s="22" t="str">
-        <x:v>eeb0bea / BLOCK-C CAPTURE.json</x:v>
+        <x:v>0841d37 · COVERAGE_LEDGER + series_sha256</x:v>
       </x:c>
       <x:c r="M26" s="22" t="str">
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ai-bots/RFC-AI-BOTS-003/BLOCK-C/CAPTURE.json</x:v>
@@ -2328,7 +2328,9 @@
       <x:c r="T26" s="22" t="str">
         <x:v>REPO_REPORT</x:v>
       </x:c>
-      <x:c r="U26" s="22" t="str"/>
+      <x:c r="U26" s="22" t="str">
+        <x:v>Cov proof, DATA_GAP fail-closed; digest de barras consumidas. 53/53 mutaciones aplicadas detectadas; otras 12 omitidas por diseño.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="31" customHeight="1">
       <x:c r="A27" s="26" t="str">
@@ -2362,10 +2364,10 @@
         <x:v>TAP-020</x:v>
       </x:c>
       <x:c r="K27" s="22" t="str">
-        <x:v>19 tests + 24 checks desde archive, no suite global</x:v>
+        <x:v>Reporte: 24 checks + 19 tests de archive para commit motor 86d4f12; captura regenerada 120 checks y 53/53 mutaciones tras fix --bars=1000. Suite global NO repetida.</x:v>
       </x:c>
       <x:c r="L27" s="22" t="str">
-        <x:v>eeb0bea / CLEAN_ARCHIVE.json</x:v>
+        <x:v>0841d37 · CLEAN_ARCHIVE.json / series_sha256</x:v>
       </x:c>
       <x:c r="M27" s="22" t="str">
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ai-bots/RFC-AI-BOTS-003/BLOCK-C/evidence/CLEAN_ARCHIVE.json</x:v>
@@ -2378,12 +2380,16 @@
       <x:c r="Q27" s="22" t="str">
         <x:v>2026-10-18</x:v>
       </x:c>
-      <x:c r="R27" s="28" t="str"/>
+      <x:c r="R27" s="28" t="str">
+        <x:v>Ejecutar clean-clone suite completa antes de certificar runtime global.</x:v>
+      </x:c>
       <x:c r="S27" s="28" t="str"/>
       <x:c r="T27" s="22" t="str">
         <x:v>REPO_REPORT</x:v>
       </x:c>
-      <x:c r="U27" s="22" t="str"/>
+      <x:c r="U27" s="22" t="str">
+        <x:v>Commits 86d4f12 (motor), eeb0bea (informe), 0841d37 (pin serie y reproducibilidad). El archivo de evidencia documenta equivalencia; los 459 tests no se reejecutaron tras cambios solo de captura/informes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="31" customHeight="1">
       <x:c r="A28" s="26" t="str">
@@ -2440,7 +2446,9 @@
       <x:c r="T28" s="22" t="str">
         <x:v>REPO_REPORT</x:v>
       </x:c>
-      <x:c r="U28" s="22" t="str"/>
+      <x:c r="U28" s="22" t="str">
+        <x:v>P0 siguiente bloque técnico: credenciales por env, recibos reales, errores, presupuesto y retries sin costes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="31" customHeight="1">
       <x:c r="A29" s="26" t="str">
@@ -4336,7 +4344,7 @@
         <x:v>PROJECT_MANAGEMENT</x:v>
       </x:c>
       <x:c r="U61" s="22" t="str">
-        <x:v>Excel maestro creado y publicado en rama independiente; no está aún en main.</x:v>
+        <x:v>Roadmap en Biblioteca y rama GitHub de gestión; cambios versionados. Se actualiza al compartir nuevo progreso, no por monitorización continua no configurada.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31" customHeight="1">
@@ -4374,10 +4382,10 @@
         <x:v>Excel binario y JSON/CSV publicados por Git blob SHA; rama independiente; merge a main pendiente</x:v>
       </x:c>
       <x:c r="L62" s="22" t="str">
-        <x:v>5f8c7610c / Excel blob 85d2f911</x:v>
+        <x:v>PR #15 · 8597750 + revisión v1.2</x:v>
       </x:c>
       <x:c r="M62" s="22" t="str">
-        <x:v>https://github.com/Extr3sao/bot_crypto/tree/project/roadmap-trading-agentic/docs/roadmap</x:v>
+        <x:v>https://github.com/Extr3sao/bot_crypto/pull/15</x:v>
       </x:c>
       <x:c r="N62" s="22" t="str">
         <x:v>ChatGPT</x:v>
@@ -4388,14 +4396,14 @@
         <x:v>2026-10-18</x:v>
       </x:c>
       <x:c r="R62" s="28" t="str">
-        <x:v>Actualizar Excel tras cada nueva fase; valorar PR a main</x:v>
+        <x:v>Actualización incremental del Excel tras cada nueva fase; valorar PR a main</x:v>
       </x:c>
       <x:c r="S62" s="28" t="str"/>
       <x:c r="T62" s="22" t="str">
         <x:v>PROJECT_MANAGEMENT</x:v>
       </x:c>
       <x:c r="U62" s="22" t="str">
-        <x:v>GitHub commit creado y objeto XLSX verificado por Git SHA-1; la integración en main aún no se ha realizado.</x:v>
+        <x:v>Excel+JSON+CSV en rama project/roadmap-trading-agentic, PR no fusionado a main. Revision v1.2 añade UX consolas invisibles.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31" customHeight="1">
@@ -4568,6 +4576,67 @@
         <x:v>REPO_REPORT</x:v>
       </x:c>
       <x:c r="U65" s="22" t="str"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>Infra &amp; experiencia Windows</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>WP-OPS-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>Eliminar ventanas visibles de bash/cmd/PowerShell al ejecutar agentes, pruebas y workers en Windows</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H66" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I66" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>TAP-044; TAP-049</x:v>
+      </x:c>
+      <x:c r="K66" t="str">
+        <x:v>0 ventanas de consola emergentes en arranque, captura, tests y cancelación; logs stdout/stderr y exit code persistidos; no procesos huérfanos ni secretos en logs</x:v>
+      </x:c>
+      <x:c r="L66" t="str">
+        <x:v>Incidencia usuario 2026-10-18: ventanas bash apareciendo mientras Codex trabaja</x:v>
+      </x:c>
+      <x:c r="M66" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/pull/15</x:v>
+      </x:c>
+      <x:c r="N66" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O66" t="str"/>
+      <x:c r="P66" t="str"/>
+      <x:c r="Q66" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R66" t="str">
+        <x:v>Inventariar lanzadores Python/Windows y shell wrappers; usar CREATE_NO_WINDOW/STARTUPINFO en procesos hijos; pruebas Windows E2E y cleanup seguro.</x:v>
+      </x:c>
+      <x:c r="S66" t="str">
+        <x:v>Origen exacto de las ventanas aún no identificado en runtime local; no cerrar por cambiar solo scripts.</x:v>
+      </x:c>
+      <x:c r="T66" t="str">
+        <x:v>USER_INCIDENT_UNVERIFIED_ROOT_CAUSE</x:v>
+      </x:c>
+      <x:c r="U66" t="str">
+        <x:v>No suprimir stdout/stderr ni esconder fallos; no matar procesos ajenos; shell=False para subprocess cuando sea viable; no desactivar shells requeridos por Codebuff/terminal integrado si no son controlables.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4627,7 +4696,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe8c59051d284d69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cdfe02cfd284344"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -4777,7 +4846,7 @@
         <x:v>PARCIAL</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>Paper y Risk canónicos, permisos; falta integrar ramas, CI y runtime map completo.</x:v>
+        <x:v>Paper y Risk canónicos, permisos; falta integrar ramas, CI y runtime map completo. Ventanas Bash Windows reportadas: raíz por verificar.</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
         <x:v>VNext</x:v>
@@ -5065,7 +5134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e944e32fe8450b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d9a2961d9ad49e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5312,10 +5381,10 @@
         <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>OPEN_GAP + riesgos y data coverage; suite afectada 459 passed</x:v>
+        <x:v>OPEN GAPS+risk y cobertura PIT; 459 tests focales previos; 120 checks/53 mutaciones regeneradas; pin datos 1000 bars</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>86d4f12 / eeb0bea</x:v>
+        <x:v>86d4f12 · 0841d37 (pines y reproducibilidad)</x:v>
       </x:c>
       <x:c r="F12" s="22" t="str">
         <x:v>TAP-020;TAP-021;TAP-022</x:v>
@@ -5480,6 +5549,32 @@
         <x:v>https://github.com/Extr3sao/bot_crypto</x:v>
       </x:c>
       <x:c r="H18" s="22" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>WP-OPS-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Windows UX</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Supresión de ventanas de terminal visible sin perder logs o exit codes; investigar launcher antes de cambiar código</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Usuario 2026-10-18</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/pull/15</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
         <x:v>2026-10-18</x:v>
       </x:c>
     </x:row>
@@ -5519,7 +5614,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d494c30861048e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5be07a99a0c045d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,6 +6124,38 @@
         <x:v>ABIERTO</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>BL-14</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Ventanas emergentes de bash/cmd/PowerShell durante ejecución automática</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>WINDOWS_UX</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>VISIBLE_CONSOLE_WINDOWS</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Usuario reporta popups; no se ha identificado aún launcher concreto</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>Redirigir stdout/stderr y ocultar ventanas de procesos hijos; probar arranque y cancelación reales</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>ABIERTO</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J2"/>
@@ -6041,7 +6168,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c6cc92555a4baa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec44e044bd44f94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6380,7 +6507,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ef5a268d4b049e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb668294728e2406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7006,6 +7133,41 @@
         <x:v>https://github.com/Extr3sao/bot_crypto/issues/14</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>EV-016</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>AI-BOTS-003C</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>SOURCE_RUNTIME_PIN</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>series_sha256 + --bars=1000 regeneración</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>0841d37</x:v>
+      </x:c>
+      <x:c r="G21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H21" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>checks</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>5 capturas con series_sha256; 24 comprobaciones por escenario, 53 mutaciones detectadas (12 no aplicadas); sin IA real.</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ai-bots/RFC-AI-BOTS-003/BLOCK-C/FINAL_REPORT.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K2"/>
@@ -7018,7 +7180,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46603a9628b47aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R040b043ac38d4df4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7206,6 +7368,52 @@
         <x:v>v1.1</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>AI-BOTS-003C</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>EVIDENCE_REPINNED</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Actualiza autoridad remota a 0841d37; series_sha256 de barras consumidas y captura con 1000 barras; 120 checks y 53 mutaciones re-verificados según informe; NO se rerun 459 tests.</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/commit/0841d372cdf36e6b52b6d8ed2e02b9d4e8c23a5e</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>v1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>USER_REPORTED_DEFECT</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Nuevo WP Windows: ningún proceso bash/cmd/PowerShell debe abrir ventana visible; conservar logs, errors y limpieza de hijos sin afectar procesos ajenos.</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Incidencia del usuario en esta conversación; raíz aún no comprobada</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>v1.2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
@@ -7213,7 +7421,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbf6ff8981204775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63a42aafe9584c52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7452,7 +7660,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>Corte GitHub: 2026-10-18 · v1.1 · Rama de gestión publicada · Sin IA real ni rentabilidad demostrada</x:v>
+        <x:v>Corte GitHub: 2026-10-18 · v1.2 · Bloque C 0841d37 · Popups bash P1 · Sin IA real ni rentabilidad demostrada</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -7491,18 +7699,15 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="B6" s="48" t="n">
-        <x:f>COUNTA(ROADMAP!A6:A65)</x:f>
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C6" s="48"/>
       <x:c r="E6" s="48" t="n">
-        <x:f>COUNTIF(ROADMAP!F6:F65,"VERIFICADO_FOCAL")</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="F6" s="48"/>
       <x:c r="H6" s="48" t="n">
-        <x:f>COUNTIF(ROADMAP!F6:F65,"PENDIENTE")+COUNTIF(ROADMAP!F6:F65,"BLOQUEADO")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="I6" s="48"/>
       <x:c r="K6" s="48" t="n">
@@ -7558,7 +7763,6 @@
         <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="L11" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K11)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
@@ -7579,7 +7783,6 @@
         <x:v>IMPLEMENTADO</x:v>
       </x:c>
       <x:c r="L12" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K12)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -7621,8 +7824,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="L14" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K14)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
@@ -7642,7 +7844,6 @@
         <x:v>PLANIFICADO</x:v>
       </x:c>
       <x:c r="L15" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K15)</x:f>
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -7663,7 +7864,6 @@
         <x:v>PROPUESTO</x:v>
       </x:c>
       <x:c r="L16" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K16)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -7815,6 +8015,6 @@
     <x:mergeCell ref="B31:I33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb7fbc5cf864af2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e9dc4d1e5794f3a"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): sync v1.3 windowless execution and external Freebuff blockers
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="Rdc0a02fb1c4f495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="Re0ec1f29096d46ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rac41de3505b14ac8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="R56293e7283804d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="Rdc34eb2ce6924743"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="Rf58241507cc4417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="R7b7d10902bfa410a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="Rcc121c59484a414b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R803f51fd71344b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="Rd1e6b932bd2b4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R40f68fd9ec4248b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rc904fbeb2f8d43a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="R54e69100cdf444cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="Rcca43954f8a649da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R2701f8e1bfd74c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="Rdd5396c657484a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="R0ca182bf6a384876"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R7c73ae9cc35b49a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -668,7 +668,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfaeb489b26294293"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R101ccd8f61494df4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1020,7 +1020,7 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>ROADMAP MAESTRO | 60 entregables</x:v>
+        <x:v>ROADMAP MAESTRO | 63 entregables</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1068,7 +1068,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>Fuente: ramas e informes GitHub (18 oct 2026). Progreso de ejecución ≠ certificación ≠ rentabilidad.</x:v>
+        <x:v>18 oct 2026 · WP-OPS-BACKGROUND-001 · windowless interno focal; Freebuff externo sigue pendiente.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -4591,16 +4591,16 @@
         <x:v>WP-OPS-BACKGROUND-001</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Eliminar ventanas visibles de bash/cmd/PowerShell al ejecutar agentes, pruebas y workers en Windows</x:v>
+        <x:v>Ejecución de Python y supervisores internos sin nuevas consolas Windows</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="G66" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H66" t="n">
-        <x:v>0</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="I66" t="n">
         <x:v>12</x:v>
@@ -4609,33 +4609,155 @@
         <x:v>TAP-044; TAP-049</x:v>
       </x:c>
       <x:c r="K66" t="str">
-        <x:v>0 ventanas de consola emergentes en arranque, captura, tests y cancelación; logs stdout/stderr y exit code persistidos; no procesos huérfanos ni secretos en logs</x:v>
+        <x:v>13 pruebas ops; 0 HIGH; 335 tests focales; logs/exit/timeout; visual NOT_OBSERVABLE</x:v>
       </x:c>
       <x:c r="L66" t="str">
-        <x:v>Incidencia usuario 2026-10-18: ventanas bash apareciendo mientras Codex trabaja</x:v>
+        <x:v>fe9b5e2 · RUN_REPORT.json · FINAL_REPORT.md</x:v>
       </x:c>
       <x:c r="M66" t="str">
-        <x:v>https://github.com/Extr3sao/bot_crypto/pull/15</x:v>
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/FINAL_REPORT.md</x:v>
       </x:c>
       <x:c r="N66" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="O66" t="str"/>
-      <x:c r="P66" t="str"/>
+      <x:c r="O66"/>
+      <x:c r="P66"/>
       <x:c r="Q66" t="str">
         <x:v>2026-10-18</x:v>
       </x:c>
       <x:c r="R66" t="str">
-        <x:v>Inventariar lanzadores Python/Windows y shell wrappers; usar CREATE_NO_WINDOW/STARTUPINFO en procesos hijos; pruebas Windows E2E y cleanup seguro.</x:v>
+        <x:v>Mantener windowless y comprobar experiencia visual después de corregir Freebuff.</x:v>
       </x:c>
       <x:c r="S66" t="str">
-        <x:v>Origen exacto de las ventanas aún no identificado en runtime local; no cerrar por cambiar solo scripts.</x:v>
+        <x:v>Freebuff Bun.spawn sin windowsHide; prueba visual NOT_OBSERVABLE; Scheduler no instalado.</x:v>
       </x:c>
       <x:c r="T66" t="str">
-        <x:v>USER_INCIDENT_UNVERIFIED_ROOT_CAUSE</x:v>
+        <x:v>REAL_RUNTIME_FOCAL</x:v>
       </x:c>
       <x:c r="U66" t="str">
-        <x:v>No suprimir stdout/stderr ni esconder fallos; no matar procesos ajenos; shell=False para subprocess cuando sea viable; no desactivar shells requeridos por Codebuff/terminal integrado si no son controlables.</x:v>
+        <x:v>Origin PE confirmado Freebuff GUI→bun CONSOLE→bash; wrapper propio CREATE_NO_WINDOW+SW_HIDE; 324 MEDIUM: 303 subprocess.run, 20 bat/cmd, 1 probe.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>TAP-062</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>Infra &amp; experiencia Windows</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>FREEBUFF-WINDOWSHIDE</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>Eliminar ventanas Bash/CMD abiertas por Freebuff/Codebuff al invocar Bun.spawn</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>BLOQUEADO</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H67" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I67" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="K67" t="str">
+        <x:v>No aparecen popups en arranque real desde Freebuff GUI; pruebas visuales independientes y logs intactos</x:v>
+      </x:c>
+      <x:c r="L67" t="str">
+        <x:v>fe9b5e2 · WINDOWLESS_EXECUTION.md · WINDOWLESS_LIVE_PROBE.json</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/docs/runtime/WINDOWLESS_EXECUTION.md</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>Proveedor Freebuff/Codebuff</x:v>
+      </x:c>
+      <x:c r="O67"/>
+      <x:c r="P67"/>
+      <x:c r="Q67" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R67" t="str">
+        <x:v>Solicitar corrección oficial de Bun.spawn con windowsHide:true; repetir prueba visual Windows.</x:v>
+      </x:c>
+      <x:c r="S67" t="str">
+        <x:v>Bun.spawn sin windowsHide en Freebuff Desktop 0.0.173; sin ajustar binarios firmados.</x:v>
+      </x:c>
+      <x:c r="T67" t="str">
+        <x:v>EXTERNAL_RUNTIME_DIAGNOSIS</x:v>
+      </x:c>
+      <x:c r="U67" t="str">
+        <x:v>Causa demostrada por cadena de padres y subsistemas PE; mitigación lanzar Freebuff desde terminal existente, no solución definitiva.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>TAP-063</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>Infra &amp; experiencia Windows</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>WP-OPS-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Activar y validar tarea programada con pythonw.exe y lanzador sin consola</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H68" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="I68" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>TAP-061</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>XML y argumentos probados; tarea instalada y ejecución visual verificada con cancelación limpia</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>fe9b5e2 · scripts/cap004_supervisor.py · RUN_REPORT.json</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/RUN_REPORT.json</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O68"/>
+      <x:c r="P68"/>
+      <x:c r="Q68" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R68" t="str">
+        <x:v>Instalación en host autorizada, test GUI de scheduler y evidencia independiente.</x:v>
+      </x:c>
+      <x:c r="S68" t="str">
+        <x:v>Tarea no registrada en Windows: modificación del host con privilegios pendiente.</x:v>
+      </x:c>
+      <x:c r="T68" t="str">
+        <x:v>IMPLEMENTED_NOT_DEPLOYED</x:v>
+      </x:c>
+      <x:c r="U68" t="str">
+        <x:v>Código y pruebas preparados, pero Task Scheduler no modificado. No desplegar sin autorización.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4696,7 +4818,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cdfe02cfd284344"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbf1e3ed81114414"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -5134,7 +5256,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d9a2961d9ad49e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R732b5d1db9844958"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5560,19 +5682,19 @@
         <x:v>Windows UX</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Supresión de ventanas de terminal visible sin perder logs o exit codes; investigar launcher antes de cambiar código</x:v>
+        <x:v>Windowless propio probado; bloqueo Freebuff externo y tarea programada sin activar</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>Usuario 2026-10-18</x:v>
+        <x:v>fe9b5e2 · FINAL_REPORT / RUN_REPORT</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>TAP-061</x:v>
+        <x:v>TAP-061;TAP-062;TAP-063</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>https://github.com/Extr3sao/bot_crypto/pull/15</x:v>
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/FINAL_REPORT.md</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>2026-10-18</x:v>
@@ -5614,7 +5736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5be07a99a0c045d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89f53e5f6d354997"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6135,25 +6257,57 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Ventanas emergentes de bash/cmd/PowerShell durante ejecución automática</x:v>
+        <x:v>Freebuff crea consola visible mediante bun.exe → bash.exe</x:v>
       </x:c>
       <x:c r="E19" t="str">
         <x:v>WINDOWS_UX</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>TAP-061</x:v>
+        <x:v>TAP-061;TAP-062</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>VISIBLE_CONSOLE_WINDOWS</x:v>
+        <x:v>EXTERNAL_WINDOWS_HIDE_MISSING</x:v>
       </x:c>
       <x:c r="H19" t="str">
-        <x:v>Usuario reporta popups; no se ha identificado aún launcher concreto</x:v>
+        <x:v>fe9b5e2: PE GUI→CONSOLE; 0 HIGH internos; visual NOT_OBSERVABLE</x:v>
       </x:c>
       <x:c r="I19" t="str">
-        <x:v>Redirigir stdout/stderr y ocultar ventanas de procesos hijos; probar arranque y cancelación reales</x:v>
+        <x:v>Corrección oficial Freebuff Bun.spawn windowsHide y test visual real</x:v>
       </x:c>
       <x:c r="J19" t="str">
-        <x:v>ABIERTO</x:v>
+        <x:v>BLOQUEADO_EXTERNO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>BL-15</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Media</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Task Scheduler sin acción pythonw/windowless instalada</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>WINDOWS_AUTOMATION</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>TAP-063</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>SCHEDULER_NOT_ACTIVATED</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>XML testeado; no se modificó la tarea programada del host</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Instalar con autorización y verificar ejecución visual y cancelación</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>PENDIENTE_AUTORIZACION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6168,7 +6322,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec44e044bd44f94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35310bbcb2349bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6507,7 +6661,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb668294728e2406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65f25b4f6ab04a57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7168,6 +7322,41 @@
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ai-bots/RFC-AI-BOTS-003/BLOCK-C/FINAL_REPORT.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>EV-017</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>WP-OPS-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>WINDOWS_RUNTIME_FOCAL</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>PE origin, pruebas Windows y captura offline vía windowless</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>fe9b5e2</x:v>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="H22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>tests failed</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>13 ops nuevos; 0 HIGH/324 MEDIUM; 9→2 adjuntos consola; visual NOT_OBSERVABLE; scheduler no registrado</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/RUN_REPORT.json</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K2"/>
@@ -7180,7 +7369,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R040b043ac38d4df4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R711939598eaf44c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7414,6 +7603,52 @@
         <x:v>v1.2</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>WP-OPS-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>IMPLEMENTED_TARGETED</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>TAP-061 corregido internamente en fe9b5e2; sin confundir pruebas estructurales con eliminación visual de popups.</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/commit/fe9b5e2623b0d023833249e9687b753eaacd27d4</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>v1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>TAP-062;TAP-063</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>EXTERNAL_AND_DEPLOYMENT_BLOCKS</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Separados el bloqueo externo Freebuff (windowsHide faltante) y tarea programada no activada.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/docs/runtime/WINDOWLESS_EXECUTION.md</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>v1.3</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
@@ -7421,7 +7656,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63a42aafe9584c52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69fac87418604ba7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7699,15 +7934,18 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="B6" s="48" t="n">
-        <x:v>61</x:v>
+        <x:f>COUNTA(ROADMAP!$A$6:$A$68)</x:f>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C6" s="48"/>
       <x:c r="E6" s="48" t="n">
-        <x:v>25</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,"VERIFICADO_FOCAL")</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F6" s="48"/>
       <x:c r="H6" s="48" t="n">
-        <x:v>19</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,"PENDIENTE")+COUNTIF(ROADMAP!$F$6:$F$68,"BLOQUEADO")</x:f>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="I6" s="48"/>
       <x:c r="K6" s="48" t="n">
@@ -7763,7 +8001,8 @@
         <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="L11" s="60" t="n">
-        <x:v>25</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K11)</x:f>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
@@ -7783,6 +8022,7 @@
         <x:v>IMPLEMENTADO</x:v>
       </x:c>
       <x:c r="L12" s="60" t="n">
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K12)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -7803,7 +8043,7 @@
         <x:v>EN_CURSO</x:v>
       </x:c>
       <x:c r="L13" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K13)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K13)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -7824,6 +8064,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="L14" s="60" t="n">
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -7844,6 +8085,7 @@
         <x:v>PLANIFICADO</x:v>
       </x:c>
       <x:c r="L15" s="60" t="n">
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K15)</x:f>
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -7864,6 +8106,7 @@
         <x:v>PROPUESTO</x:v>
       </x:c>
       <x:c r="L16" s="60" t="n">
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K16)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -7884,8 +8127,8 @@
         <x:v>BLOQUEADO</x:v>
       </x:c>
       <x:c r="L17" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K17)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K17)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
@@ -7893,7 +8136,7 @@
         <x:v>RECHAZADO</x:v>
       </x:c>
       <x:c r="L18" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$65,K18)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K18)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -8015,6 +8258,6 @@
     <x:mergeCell ref="B31:I33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e9dc4d1e5794f3a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9bf33e0e6c848fe"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): v1.4 market data RFC005, incremental intelligence and fetch audit
- Extend master tracker TAP-064..TAP-071 (71 items), BL-16/17, historical registry and mirror
- Add source-grounded RFC, audit, Codex prompt, roadmap delta and download classification matrix
- No runtime, scheduler, AI API or risk changes
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="Rd1e6b932bd2b4d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R40f68fd9ec4248b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="Rc904fbeb2f8d43a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="R54e69100cdf444cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="Rcca43954f8a649da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R2701f8e1bfd74c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="Rdd5396c657484a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="R0ca182bf6a384876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R7c73ae9cc35b49a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROADMAP" sheetId="1" r:id="R146e1cd24c58412e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="2" r:id="R2d3ff3103b564163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFC_Y_WP" sheetId="3" r:id="R6da27da9bd9b4eac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLOQUEOS" sheetId="4" r:id="Rff0d5ce5b453448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPENDENCIAS" sheetId="5" r:id="R0680f05b634f418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCIAS" sheetId="6" r:id="R8fcef66ce8ae4096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HISTORIAL" sheetId="7" r:id="Rcbb2f1d072764147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO_ACTUALIZAR" sheetId="8" r:id="R6c141424a8fe4ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="9" r:id="R31941b476338477f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -668,7 +668,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R101ccd8f61494df4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1f11a02e2104f26"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1020,7 +1020,7 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>ROADMAP MAESTRO | 63 entregables</x:v>
+        <x:v>ROADMAP MAESTRO | 71 entregables</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1068,7 +1068,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>18 oct 2026 · WP-OPS-BACKGROUND-001 · windowless interno focal; Freebuff externo sigue pendiente.</x:v>
+        <x:v>18 oct 2026 · v1.4 · RFC-TAP-MARKET-005 · data incremental + IA event-driven; P0 auditar origen de fetches.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -4758,6 +4758,494 @@
       </x:c>
       <x:c r="U68" t="str">
         <x:v>Código y pruebas preparados, pero Task Scheduler no modificado. No desplegar sin autorización.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>TAP-064</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>Datos de mercado</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005A</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Atribuir fetch_ohlcv y tareas reales a PID/PPID, owner, consumidor y run_id</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H69" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I69" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>TAP-061; TAP-063</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>Correlación proceso→task→req_id→caller→uso, o UNKNOWN sin falsos éxitos</x:v>
+      </x:c>
+      <x:c r="L69" t="str">
+        <x:v>Revisión GitHub fe9b5e2; screenshot fetch_ohlcv; fetch limits 1000/500/500</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O69"/>
+      <x:c r="P69"/>
+      <x:c r="Q69" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R69" t="str">
+        <x:v>WP-005A: Get-ScheduledTask read-only y mapa de entrypoints; no modificar tasks.</x:v>
+      </x:c>
+      <x:c r="S69" t="str">
+        <x:v>No existe todavía evidencia PID/task/run_id que atribuya esa descarga concreta.</x:v>
+      </x:c>
+      <x:c r="T69" t="str">
+        <x:v>SOURCE_AUDIT_PENDING_RUNTIME</x:v>
+      </x:c>
+      <x:c r="U69" t="str">
+        <x:v>CCXTExchangeConnector emite logs; real_market_context coincide en límites, pero la fuente de la captura no está identificada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>TAP-065</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>Datos de mercado</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005B</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Medir coste y cobertura de recargas de históricos 1h/4h/1d y readers actuales</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H70" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I70" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>TAP-064</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>Misma ventana/activos; requests/h, bytes, age, duplicate, gap, lag, proveedor, destino y consumo</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>RFC-TAP-MARKET-005 / source baseline (NO RUN)</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N70" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O70"/>
+      <x:c r="P70"/>
+      <x:c r="Q70" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R70" t="str">
+        <x:v>Obtener baseline de varios ciclos y distinguir bootstrap de recarga frecuente.</x:v>
+      </x:c>
+      <x:c r="S70" t="str">
+        <x:v>Tasa real de peticiones y uso de cache no medida; no afirmar redundancia aún.</x:v>
+      </x:c>
+      <x:c r="T70" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U70" t="str">
+        <x:v>No convertir coincidencia de logs en causalidad de Task Scheduler; no apagar procesos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>TAP-066</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Datos de mercado</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>03 Runtime Authority</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005C</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Bootstrapping limitado e ingestión incremental con watermark y correcciones</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>PLANIFICADO</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H71" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I71" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>TAP-065</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>Mismos datos finales que baseline con menos llamadas; reinicio idempotente, no HTF futuro</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>RFC-005 WP plan; adapters existentes OHLCVFetcher/Store</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O71"/>
+      <x:c r="P71"/>
+      <x:c r="Q71" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R71" t="str">
+        <x:v>Implementar delta-reader reutilizando CCXT/store y cuotas; RED→GREEN.</x:v>
+      </x:c>
+      <x:c r="S71" t="str">
+        <x:v>No activar sin demostrar equivalencia de datos y fuente.</x:v>
+      </x:c>
+      <x:c r="T71" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U71" t="str">
+        <x:v>No instalar colector adicional ni copiar framework de terceros; un owner lógico.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>TAP-067</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>Market Intelligence</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>06 Market Intelligence</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005D</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>MarketSnapshot causal para bots visual/contextual y runtime PAPER/SHADOW</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>PLANIFICADO</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I72" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>TAP-066; TAP-022; TAP-024</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>PIT, fecha disponibilidad, freshness, hash y consumo real; RiskManager/Admission intactos</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>RFC-005 snapshot contract</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O72"/>
+      <x:c r="P72"/>
+      <x:c r="Q72" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R72" t="str">
+        <x:v>Conectar snapshot validado a eventos del runtime sin bypass de estrategia.</x:v>
+      </x:c>
+      <x:c r="S72" t="str">
+        <x:v>Coleccionista WebSocket solo DISCOVERY y estrategia PAPER no admitida.</x:v>
+      </x:c>
+      <x:c r="T72" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U72" t="str">
+        <x:v>Datos cerrados &gt; datos recibidos; sin snapshot FRESH bloquear propuesta de entrada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>TAP-068</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>Market Intelligence</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>09 Decision/Critic</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005E</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Disparadores IA por evento de mercado y cuotas, deduplicación y control de costes</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>PLANIFICADO</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H73" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I73" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>TAP-067; TAP-023; TAP-025</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>Un evento válido→como máximo una petición autorizada; sin clave/budget=0→cero llamadas</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>RFC-005 event trigger plan</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O73"/>
+      <x:c r="P73"/>
+      <x:c r="Q73" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R73" t="str">
+        <x:v>Probar offline triggers de cierre/regime-change sin LLM de pago ni requests inventados.</x:v>
+      </x:c>
+      <x:c r="S73" t="str">
+        <x:v>REAL_MODEL_CALLED=false; Freebuff no es provider programático demostrado.</x:v>
+      </x:c>
+      <x:c r="T73" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U73" t="str">
+        <x:v>LLM analiza snapshots filtrados; market data API ≠ inferencia LLM; nunca invocar cada tick.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>TAP-069</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Datos de mercado</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>12 Observabilidad</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005F</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Clasificar redundancias y proponer desactivaciones seguras por evidencia</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>PLANIFICADO</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H74" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I74" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>TAP-064; TAP-065; TAP-066</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>KEEP/OPTIMIZE/MERGE/DISABLE_CANDIDATE + compatibilidad, ahorro y rollback</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>RFC-005 decision matrix</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O74"/>
+      <x:c r="P74"/>
+      <x:c r="Q74" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R74" t="str">
+        <x:v>Probar equivalencia A/B y preparar matriz sin deshabilitar tareas existentes.</x:v>
+      </x:c>
+      <x:c r="S74" t="str">
+        <x:v>Desactivaciones requieren identificación y autorización operativa del host.</x:v>
+      </x:c>
+      <x:c r="T74" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U74" t="str">
+        <x:v>No borrar campañas ni OOS históricos ni tareas desconocidas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>TAP-070</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>Datos de mercado</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>12 Observabilidad</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005G</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>Verificar de modo independiente ingestión PIT, continuidad y triggers de IA</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>PLANIFICADO</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I75" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>TAP-066; TAP-067; TAP-068</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>Builder != Verifier, mutaciones PIT/huecos/doble scheduler/disk, run report y clean checkout</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>RFC-005 acceptance ACC01..ACC16</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="O75"/>
+      <x:c r="P75"/>
+      <x:c r="Q75" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R75" t="str">
+        <x:v>Crear verifier independiente y ejecutar mismo runtime que producción PAPER.</x:v>
+      </x:c>
+      <x:c r="S75" t="str">
+        <x:v>Suite global histórica 14 FAIL; no presentar PASS global hasta reejecutar.</x:v>
+      </x:c>
+      <x:c r="T75" t="str">
+        <x:v>DESIGN_ONLY</x:v>
+      </x:c>
+      <x:c r="U75" t="str">
+        <x:v>No certificar por solo tests de fixture o mock; fallo de integridad fail-closed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>TAP-071</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>Operaciones Windows</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>14 Paper</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>RFC-TAP-MARKET-005 / 005H</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Activación opcional de adquisición incremental supervisada en PAPER sin Freebuff</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>BLOQUEADO</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H76" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I76" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>TAP-070; TAP-062; TAP-063</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>Una sola vía programada con owner, logs, prueba de rollback y cero popups del proceso propio</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>RFC-005 WP-005H activation gate</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>Usuario + Codex</x:v>
+      </x:c>
+      <x:c r="O76"/>
+      <x:c r="P76"/>
+      <x:c r="Q76" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="R76" t="str">
+        <x:v>Solo tras permiso para modificar Task Scheduler, verificación e inventario de tareas existentes.</x:v>
+      </x:c>
+      <x:c r="S76" t="str">
+        <x:v>Cambios a tareas reales/host requieren aprobación; popups Freebuff siguen externos.</x:v>
+      </x:c>
+      <x:c r="T76" t="str">
+        <x:v>PROPOSED_DEPLOYMENT_GATE</x:v>
+      </x:c>
+      <x:c r="U76" t="str">
+        <x:v>Preparación offline permitida; no activar ni deshabilitar programas sin consentimiento.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4818,7 +5306,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbf1e3ed81114414"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3587323a529842e3"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -5256,7 +5744,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R732b5d1db9844958"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re432b6d884fb47a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5697,6 +6185,32 @@
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/FINAL_REPORT.md</x:v>
       </x:c>
       <x:c r="H19" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>RFC-TAP-MARKET-005</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Market Data &amp; AI</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>PROPUESTO</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Auditoría de recargas 1000/500/500 + incremental PIT + triggers IA por evento; despliegue solo autorizado</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>RFC + auditoría + issue #16 (sin código ni runtime nuevo)</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>TAP-064..TAP-071</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
         <x:v>2026-10-18</x:v>
       </x:c>
     </x:row>
@@ -5736,7 +6250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89f53e5f6d354997"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6d4f83b78b74817"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6310,6 +6824,70 @@
         <x:v>PENDIENTE_AUTORIZACION</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>BL-16</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Origen exacto de descargas 1000/500/500 no atribuido al proceso/tarea</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>MARKET_DATA</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>TAP-064; TAP-065</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>FETCH_ORIGIN_NOT_ATTRIBUTED</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>CCXT log y limits real_market_context coinciden; PID/caller/task aún UNKNOWN</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>WP-005A inspección solo lectura + correlación req_id→consumer</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>ABIERTO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>BL-17</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Datos de market no integrados de forma incremental ni en inferencia LLM real</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>DATA_TO_AI</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>TAP-066;TAP-067;TAP-068</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>NO_PROSPECTIVE_AI_DATA_PIPELINE</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Collector WebSocket DISCOVERY; AI-BOTS-003C replay; REAL_MODEL_CALLED=false</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>WP-005B..005G; autorizaciones proveedor/gasto para real LLM</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>ABIERTO</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J2"/>
@@ -6322,7 +6900,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35310bbcb2349bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41094e64e5cd4427"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6654,6 +7232,76 @@
         <x:v>Baseline pérdidas exige nuevos experimentos</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>TAP-066</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>TAP-065</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>No optimizar sin baseline request/data equivalence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>TAP-067</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>TAP-066</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Snapshots PIT requieren deltas válidos y cobertura</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>TAP-068</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>TAP-067</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>IA event-driven solo consume snapshots causales</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>TAP-070</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>TAP-068</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Verificar triggers, esquema y proveedor offline</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>TAP-071</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>TAP-070</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Operativa con aprobación</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>Modificar tarea real solo tras verificación y consentimiento</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D2"/>
@@ -6661,7 +7309,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65f25b4f6ab04a57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2e9fe503d854b2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7357,6 +8005,41 @@
         <x:v>https://github.com/Extr3sao/bot_crypto/blob/agent/ai-bots/RFC-TAP-AI-BOTS-003/reports/ops/WP-OPS-BACKGROUND-001/RUN_REPORT.json</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>EV-018</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>RFC-TAP-MARKET-005</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>SOURCE_CORRELATION_ONLY</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Screenshot CCXT fetch_ohlcv + patrón 1000/500/500</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>fe9b5e2</x:v>
+      </x:c>
+      <x:c r="G23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>WPs executed</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Análisis código CCXT y real_market_context; caller PID/task UNKNOWN; no nueva descarga ejecutada por RFC-005</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K2"/>
@@ -7369,7 +8052,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R711939598eaf44c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22feb76d452f4282"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7649,6 +8332,29 @@
         <x:v>v1.3</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>RFC-TAP-MARKET-005</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>PROPOSED_REGISTERED</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Se añaden TAP-064..071, BL-16/17; separar descargas de precios del proveedor IA; ninguna task tocada.</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>https://github.com/Extr3sao/bot_crypto/issues/16</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>v1.4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
@@ -7656,7 +8362,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69fac87418604ba7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb25a67fad6964a53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7934,18 +8640,18 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="B6" s="48" t="n">
-        <x:f>COUNTA(ROADMAP!$A$6:$A$68)</x:f>
-        <x:v>63</x:v>
+        <x:f>COUNTA(ROADMAP!$A$6:$A$76)</x:f>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C6" s="48"/>
       <x:c r="E6" s="48" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,"VERIFICADO_FOCAL")</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,"VERIFICADO_FOCAL")</x:f>
         <x:v>26</x:v>
       </x:c>
       <x:c r="F6" s="48"/>
       <x:c r="H6" s="48" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,"PENDIENTE")+COUNTIF(ROADMAP!$F$6:$F$68,"BLOQUEADO")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,"PENDIENTE")+COUNTIF(ROADMAP!$F$6:$F$76,"BLOQUEADO")</x:f>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I6" s="48"/>
       <x:c r="K6" s="48" t="n">
@@ -7989,19 +8695,19 @@
         <x:v>P0 · 01</x:v>
       </x:c>
       <x:c r="C11" s="22" t="str">
-        <x:v>Provider receipts offline + budget/retries</x:v>
+        <x:v>Identificar proceso/tarea que descarga velas</x:v>
       </x:c>
       <x:c r="D11" s="22" t="str">
-        <x:v>TAP-023</x:v>
+        <x:v>TAP-064/065</x:v>
       </x:c>
       <x:c r="E11" s="22" t="str">
-        <x:v>Sin credencial/gasto por ahora</x:v>
+        <x:v>Sin atribución no se desactiva nada</x:v>
       </x:c>
       <x:c r="K11" s="62" t="str">
         <x:v>VERIFICADO_FOCAL</x:v>
       </x:c>
       <x:c r="L11" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K11)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K11)</x:f>
         <x:v>26</x:v>
       </x:c>
     </x:row>
@@ -8010,19 +8716,19 @@
         <x:v>P0 · 02</x:v>
       </x:c>
       <x:c r="C12" s="22" t="str">
-        <x:v>Feed 1m/tick + captura prospectiva continua</x:v>
+        <x:v>Datos incrementales y snapshots PIT</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>TAP-024 / TAP-049</x:v>
+        <x:v>TAP-066/067</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>Causalidad sub-vela y scheduler</x:v>
+        <x:v>Bootstrapping once; no futuras HTF</x:v>
       </x:c>
       <x:c r="K12" s="64" t="str">
         <x:v>IMPLEMENTADO</x:v>
       </x:c>
       <x:c r="L12" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K12)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K12)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -8031,19 +8737,19 @@
         <x:v>P0 · 03</x:v>
       </x:c>
       <x:c r="C13" s="22" t="str">
-        <x:v>Resolver 14 FAIL globales y CI clean</x:v>
+        <x:v>Proveedor IA offline + receipts</x:v>
       </x:c>
       <x:c r="D13" s="22" t="str">
-        <x:v>TAP-048</x:v>
+        <x:v>TAP-023 / 068</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
-        <x:v>No proclamar PASS global</x:v>
+        <x:v>Sin clave/coste → 0 llamadas</x:v>
       </x:c>
       <x:c r="K13" s="66" t="str">
         <x:v>EN_CURSO</x:v>
       </x:c>
       <x:c r="L13" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K13)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K13)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -8052,41 +8758,41 @@
         <x:v>P0 · 04</x:v>
       </x:c>
       <x:c r="C14" s="22" t="str">
-        <x:v>Admisión de estrategia con OOS neto</x:v>
+        <x:v>Feed prospectivo y continuidad</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
-        <x:v>TAP-035 / TAP-041</x:v>
+        <x:v>TAP-024/049</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
-        <x:v>0 estrategias admitidas</x:v>
+        <x:v>1m/quotes; datos observables</x:v>
       </x:c>
       <x:c r="K14" s="68" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="L14" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K14)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K14)</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="B15" s="55" t="str">
-        <x:v>P1 · 05</x:v>
+        <x:v>P0 · 05</x:v>
       </x:c>
       <x:c r="C15" s="22" t="str">
-        <x:v>REA + BOT-CRI-01 crítico solo SHADOW</x:v>
+        <x:v>Resolver CI full y gate PAPER</x:v>
       </x:c>
       <x:c r="D15" s="22" t="str">
-        <x:v>TAP-028 / TAP-030</x:v>
+        <x:v>TAP-048 / 035</x:v>
       </x:c>
       <x:c r="E15" s="22" t="str">
-        <x:v>Sin bloquear fills</x:v>
+        <x:v>No saltar admisión ni 14 FAIL históricos</x:v>
       </x:c>
       <x:c r="K15" s="70" t="str">
         <x:v>PLANIFICADO</x:v>
       </x:c>
       <x:c r="L15" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K15)</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K15)</x:f>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
@@ -8106,7 +8812,7 @@
         <x:v>PROPUESTO</x:v>
       </x:c>
       <x:c r="L16" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K16)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K16)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -8127,8 +8833,8 @@
         <x:v>BLOQUEADO</x:v>
       </x:c>
       <x:c r="L17" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K17)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K17)</x:f>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
@@ -8136,7 +8842,7 @@
         <x:v>RECHAZADO</x:v>
       </x:c>
       <x:c r="L18" s="60" t="n">
-        <x:f>COUNTIF(ROADMAP!$F$6:$F$68,K18)</x:f>
+        <x:f>COUNTIF(ROADMAP!$F$6:$F$76,K18)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -8258,6 +8964,6 @@
     <x:mergeCell ref="B31:I33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9bf33e0e6c848fe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e5d71891d0f4acf"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): v1.7 — cierre de la sincronización LOCAL -> GITHUB y re-medida de gates
Actualiza JSON + CSV + XLSX en el mismo commit (regla del propio README): TAP-072
(35/35 ramas publicadas, 0 commits sin publicar, 4 reportes publicados), TAP-073
(re-medición 2026-10-26: ruff 130 / format 444 / mypy 297 idénticos a v1.6 y
pytest 79F/3274P/34S/14E, 19 de 20 ficheros coincidentes con la baseline),
TAP-075 (31 PR draft, #19-#35 y #36-#49) y TAP-076 (colección rota re-verificada).
Nada pasa a CERTIFIED por publicar.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -1154,7 +1154,7 @@
     <row r="3" ht="24" customHeight="1" s="82">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>25 oct 2026 · v1.6 · sincronización LOCAL -&gt; GITHUB</t>
+          <t>2026-10-26 · v1.7 · sincronización LOCAL -&gt; GITHUB cerrada: 35/35 ramas publicadas, 31 PR draft, gates en rojo preexistente</t>
         </is>
       </c>
       <c r="B3" s="1" t="n"/>
@@ -7553,12 +7553,12 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>0 commits locales sin publicar; 18 ramas con SHA local == SHA remoto; respaldo SHA-256 previo a tocar Git</t>
+          <t>0 commits locales sin publicar (git rev-list --branches --not --remotes=origin = 0); 35/35 ramas con SHA local == SHA remoto; respaldo SHA-256 previo a tocar Git</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>5b63f265 / LOCAL_GITHUB_SYNC_AUDIT.md + FINAL_GITHUB_SYNC_REPORT.md</t>
+          <t>5b63f265 / LOCAL_GITHUB_SYNC_AUDIT.md + .json + FINAL_GITHUB_SYNC_REPORT.md + .json + EXCLUDED_FROM_SYNC_MANIFEST.json (publicados en GitHub)</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -7573,12 +7573,12 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Revisar y cerrar los PR draft #19-#35</t>
+          <t>Revisar y cerrar los 31 PR draft (#19-#35 y #36-#49)</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -7588,7 +7588,7 @@
       </c>
       <c r="U77" t="inlineStr">
         <is>
-          <t>SYNC_COMPLETE != MAIN_INTEGRATED != RUNTIME_CERTIFIED != PROFITABLE. Sin reset --hard, clean -fd, push --force ni rebase; ningún worktree, rama, stash o evidencia borrado.</t>
+          <t>SYNC_COMPLETE != MAIN_INTEGRATED != RUNTIME_CERTIFIED != PROFITABLE. Sin reset --hard, clean -fd, push --force ni rebase; ningún worktree, rama, stash o evidencia borrado. v1.7: los cuatro reportes de sincronización se publicaron en la rama sync/uncommitted-main-20261025 (PR #19); 14 ramas de preservación recibieron PR #36-#49.</t>
         </is>
       </c>
     </row>
@@ -7641,12 +7641,12 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>ruff check 130 errores y ruff format 444 ficheros en e67194e7; mypy 297 errores; pytest 90 failed / 3263 passed / 14 errors</t>
+          <t>ruff check 130 errores y ruff format 444 ficheros en e67194e7; mypy 297 errores; pytest 79 failed / 3274 passed / 34 skipped / 14 errors</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>checkout limpio de e67194e7 (ff-wt-main001), uv sync --frozen, 2026-10-25</t>
+          <t>checkout limpio gate-main-20261026 de e67194e7 con PYTHONPATH al src limpio, 2026-10-26; ruff/format/mypy idénticos a los de v1.6 (2026-10-25, 90 failed / 3263 passed)</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -7661,7 +7661,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="U78" t="inlineStr">
         <is>
-          <t>Falla preexistente: NO la introduce la sincronización. origin/main 5e6f9632 sí está en verde (ruff/mypy/format y 582 tests PASS), pero está 263 commits por detrás del linaje local.</t>
+          <t>Falla preexistente: NO la introduce la sincronización. Re-medición 2026-10-26: mismos 130/444/297 que en v1.6 y 19 de 20 ficheros con fallos coinciden con la baseline (tests/unit/research/**). La CI Baseline ya fallaba sobre origin/main desde 2026-07-10. origin/main 5e6f9632 sí está en verde (582 tests PASS) pero está 263 commits por detrás.</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>17 PR draft abiertos (#19-#35); cabeceras == SHA de rama local</t>
+          <t>31 PR draft abiertos (#19-#35 y #36-#49); cabeceras == SHA de rama local</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>refs/pull/19..35/head verificados con git ls-remote</t>
+          <t>refs/pull/*/head verificados con git ls-remote y API /pulls?state=open (38 PR abiertos)</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>Todos en draft: gates NO ejecutados en esas ramas -&gt; NOT_VERIFIED. audit/economic-blocker-001 no recibe PR porque es idéntica a main.</t>
+          <t>Todos en draft: gates NO ejecutados en esas ramas -&gt; NOT_VERIFIED. audit/economic-blocker-001 no recibe PR porque es idéntica a main; main se integra a través del PR #18.</t>
         </is>
       </c>
     </row>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>8 commits en rama sync/uncommitted-main-20261025; árbol limpio; PR #19 draft</t>
+          <t>8 commits en rama sync/uncommitted-main-20261025; árbol limpio; PR #19 draft; colección rota re-verificada 2026-10-26 (3532 tests + 1 error de import)</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7960,7 +7960,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>El shim de settings.py (346 -&gt; 27 lineas) rompe la recolección: tests/unit/config/test_failfast.py no puede importar YamlDirectorySource. Publicado, NO integrado.</t>
+          <t>El shim de settings.py (346 -&gt; 27 lineas) rompe la recolección: tests/unit/config/test_failfast.py no puede importar YamlDirectorySource (commit c16c241b). Publicado, NO integrable. La colección de main e67194e7 sí es correcta (3401 tests, 0 errores).</t>
         </is>
       </c>
     </row>
@@ -12283,7 +12283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" style="82" min="1" max="1"/>
@@ -12809,6 +12809,43 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>v1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>v1.7 — sincronización LOCAL -&gt; GITHUB cerrada</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>35/35 ramas publicadas y verificadas, 0 commits sin publicar, 31 PR draft (#19-#49), 4 reportes publicados</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TAP-072, TAP-073, TAP-075, TAP-076</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Gates re-meditos: ruff 130 / format 444 / mypy 297 / pytest 79F-3274P-14E (preexistente)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Codebuff</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SYNC_COMPLETE != MAIN_INTEGRATED != RUNTIME_CERTIFIED != PROFITABLE</t>
         </is>
       </c>
     </row>
@@ -13135,7 +13172,7 @@
     <row r="3" ht="24" customHeight="1" s="82">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Corte GitHub: 2026-10-25 · v1.6 · 18 ramas publicadas, 17 PR draft · origin/main 263 commits atrás · sin IA real ni rentabilidad demostrada</t>
+          <t>Corte GitHub: 2026-10-26 · v1.7 · 0 commits sin publicar · 31 PR draft · origin/main 263 commits por detrás</t>
         </is>
       </c>
       <c r="B3" s="1" t="n"/>
@@ -13213,8 +13250,6 @@
       <c r="K7" s="1" t="n"/>
       <c r="L7" s="1" t="n"/>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10" ht="28" customHeight="1" s="82">
       <c r="B10" s="53" t="inlineStr">
         <is>
@@ -13467,7 +13502,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="28" customHeight="1" s="82">
       <c r="B20" s="53" t="inlineStr">
         <is>
@@ -13566,9 +13600,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="B31" s="86" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(roadmap): v1.7 — cifras de cierre 36/36 ramas y commit de los informes
TAP-072 pasa de 35/35 a 36/36 ramas con SHA local == SHA remoto (se suma
feat/wp-signal-001-003, de un agente paralelo), fija los 40 tags sync/orphan-*
y apunta como evidencia el commit 6381c9f7 que publica los cuatro reportes.
JSON + CSV + XLSX actualizados en el mismo commit, como exige el README.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
+++ b/docs/roadmap/ROADMAP_TRADING_AGENTIC_PORTABLE.xlsx
@@ -7553,12 +7553,12 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>0 commits locales sin publicar (git rev-list --branches --not --remotes=origin = 0); 35/35 ramas con SHA local == SHA remoto; respaldo SHA-256 previo a tocar Git</t>
+          <t>0 commits locales sin publicar (git rev-list --branches --not --remotes=origin = 0); 36/36 ramas con SHA local == SHA remoto (35 de la sincronización + feat/wp-signal-001-003 de un agente paralelo); 40 tags sync/orphan-*; respaldo SHA-256 previo a tocar Git</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>5b63f265 / LOCAL_GITHUB_SYNC_AUDIT.md + .json + FINAL_GITHUB_SYNC_REPORT.md + .json + EXCLUDED_FROM_SYNC_MANIFEST.json (publicados en GitHub)</t>
+          <t>6381c9f7 / LOCAL_GITHUB_SYNC_AUDIT.md + .json + FINAL_GITHUB_SYNC_REPORT.md + .json + EXCLUDED_FROM_SYNC_MANIFEST.json (publicados en GitHub)</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">

</xml_diff>